<commit_message>
Update user specification Excel file
</commit_message>
<xml_diff>
--- a/data/user_specification_excel_folder/user_specification.xlsx
+++ b/data/user_specification_excel_folder/user_specification.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,7 +486,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -509,7 +509,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">

</xml_diff>